<commit_message>
test(login): TC02 Để trống cả hai ô (PASS)
</commit_message>
<xml_diff>
--- a/outputs/Login-Test-Cases.xlsx
+++ b/outputs/Login-Test-Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="Rafb2c4fdc4434198"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R7b6eda34fe984611"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -426,9 +426,11 @@
         <x:v>Ở lại login và hiển thị thông báo từ chối hoặc yêu cầu nhập dữ liệu.</x:v>
       </x:c>
       <x:c r="G8" s="9" t="str">
-        <x:v>NOT RUN</x:v>
-      </x:c>
-      <x:c r="H8" s="9" t="str"/>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H8" s="9" t="str">
+        <x:v>Đã chạy trên Chrome hiển thị; các assertion đạt.</x:v>
+      </x:c>
       <x:c r="I8" s="9" t="str">
         <x:v>artifacts/TC02.png; Allure/TC02</x:v>
       </x:c>

</xml_diff>

<commit_message>
test(login): TC03 Thiếu tên đăng nhập (PASS)
</commit_message>
<xml_diff>
--- a/outputs/Login-Test-Cases.xlsx
+++ b/outputs/Login-Test-Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R7b6eda34fe984611"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R422835d423364ffc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -455,9 +455,11 @@
         <x:v>Ở lại login và hiển thị thông báo từ chối hoặc yêu cầu nhập dữ liệu.</x:v>
       </x:c>
       <x:c r="G9" s="9" t="str">
-        <x:v>NOT RUN</x:v>
-      </x:c>
-      <x:c r="H9" s="9" t="str"/>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H9" s="9" t="str">
+        <x:v>Đã chạy trên Chrome hiển thị; các assertion đạt.</x:v>
+      </x:c>
       <x:c r="I9" s="9" t="str">
         <x:v>artifacts/TC03.png; Allure/TC03</x:v>
       </x:c>

</xml_diff>

<commit_message>
test(login): TC04 Thiếu mật khẩu (PASS)
</commit_message>
<xml_diff>
--- a/outputs/Login-Test-Cases.xlsx
+++ b/outputs/Login-Test-Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R422835d423364ffc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R0d4047188048472f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -484,9 +484,11 @@
         <x:v>Ở lại login và hiển thị thông báo từ chối hoặc yêu cầu nhập dữ liệu.</x:v>
       </x:c>
       <x:c r="G10" s="9" t="str">
-        <x:v>NOT RUN</x:v>
-      </x:c>
-      <x:c r="H10" s="9" t="str"/>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H10" s="9" t="str">
+        <x:v>Đã chạy trên Chrome hiển thị; các assertion đạt.</x:v>
+      </x:c>
       <x:c r="I10" s="9" t="str">
         <x:v>artifacts/TC04.png; Allure/TC04</x:v>
       </x:c>

</xml_diff>

<commit_message>
test(login): TC05 Tài khoản không tồn tại (PASS)
</commit_message>
<xml_diff>
--- a/outputs/Login-Test-Cases.xlsx
+++ b/outputs/Login-Test-Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R0d4047188048472f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="Rd6dd148a73e04f2f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -513,9 +513,11 @@
         <x:v>Ở lại login và hiển thị thông báo từ chối thông tin không hợp lệ.</x:v>
       </x:c>
       <x:c r="G11" s="9" t="str">
-        <x:v>NOT RUN</x:v>
-      </x:c>
-      <x:c r="H11" s="9" t="str"/>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H11" s="9" t="str">
+        <x:v>Đã chạy trên Chrome hiển thị; các assertion đạt.</x:v>
+      </x:c>
       <x:c r="I11" s="9" t="str">
         <x:v>artifacts/TC05.png; Allure/TC05</x:v>
       </x:c>

</xml_diff>

<commit_message>
test(login): TC06 Bật và tắt giữ đăng nhập (PASS)
</commit_message>
<xml_diff>
--- a/outputs/Login-Test-Cases.xlsx
+++ b/outputs/Login-Test-Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="Rd6dd148a73e04f2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R3bf20afe4dd245e0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -542,9 +542,11 @@
         <x:v>Checkbox lần lượt false, true, false; không submit form.</x:v>
       </x:c>
       <x:c r="G12" s="9" t="str">
-        <x:v>NOT RUN</x:v>
-      </x:c>
-      <x:c r="H12" s="9" t="str"/>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H12" s="9" t="str">
+        <x:v>Đã chạy trên Chrome hiển thị; các assertion đạt.</x:v>
+      </x:c>
       <x:c r="I12" s="9" t="str">
         <x:v>artifacts/TC06.png; Allure/TC06</x:v>
       </x:c>

</xml_diff>

<commit_message>
chore: finalize Allure 3 reporting and verified Excel results
</commit_message>
<xml_diff>
--- a/outputs/Login-Test-Cases.xlsx
+++ b/outputs/Login-Test-Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R3bf20afe4dd245e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R18073f1d7e2f4bf4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -377,7 +377,7 @@
         <x:v>Bằng chứng</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="108" customHeight="1">
+    <x:row r="7" ht="66" customHeight="1">
       <x:c r="A7" s="9" t="str">
         <x:v>TC01</x:v>
       </x:c>
@@ -406,7 +406,7 @@
         <x:v>artifacts/TC01.png; Allure/TC01</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="108" customHeight="1">
+    <x:row r="8" ht="66" customHeight="1">
       <x:c r="A8" s="9" t="str">
         <x:v>TC02</x:v>
       </x:c>
@@ -429,13 +429,13 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="H8" s="9" t="str">
-        <x:v>Đã chạy trên Chrome hiển thị; các assertion đạt.</x:v>
+        <x:v>Bạn chưa nhập tên đăng nhập</x:v>
       </x:c>
       <x:c r="I8" s="9" t="str">
         <x:v>artifacts/TC02.png; Allure/TC02</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="108" customHeight="1">
+    <x:row r="9" ht="66" customHeight="1">
       <x:c r="A9" s="9" t="str">
         <x:v>TC03</x:v>
       </x:c>
@@ -458,13 +458,13 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="H9" s="9" t="str">
-        <x:v>Đã chạy trên Chrome hiển thị; các assertion đạt.</x:v>
+        <x:v>Bạn chưa nhập tên đăng nhập</x:v>
       </x:c>
       <x:c r="I9" s="9" t="str">
         <x:v>artifacts/TC03.png; Allure/TC03</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="108" customHeight="1">
+    <x:row r="10" ht="66" customHeight="1">
       <x:c r="A10" s="9" t="str">
         <x:v>TC04</x:v>
       </x:c>
@@ -487,13 +487,13 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="H10" s="9" t="str">
-        <x:v>Đã chạy trên Chrome hiển thị; các assertion đạt.</x:v>
+        <x:v>Bạn chưa nhập mật khẩu</x:v>
       </x:c>
       <x:c r="I10" s="9" t="str">
         <x:v>artifacts/TC04.png; Allure/TC04</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="108" customHeight="1">
+    <x:row r="11" ht="66" customHeight="1">
       <x:c r="A11" s="9" t="str">
         <x:v>TC05</x:v>
       </x:c>
@@ -516,13 +516,13 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="H11" s="9" t="str">
-        <x:v>Đã chạy trên Chrome hiển thị; các assertion đạt.</x:v>
+        <x:v>Tài khoản hoặc mật khẩu không đúng.</x:v>
       </x:c>
       <x:c r="I11" s="9" t="str">
         <x:v>artifacts/TC05.png; Allure/TC05</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="108" customHeight="1">
+    <x:row r="12" ht="66" customHeight="1">
       <x:c r="A12" s="9" t="str">
         <x:v>TC06</x:v>
       </x:c>

</xml_diff>

<commit_message>
test(login): TC07 Chuyển từ username sang password bằng Tab (BLOCKED)
</commit_message>
<xml_diff>
--- a/outputs/Login-Test-Cases.xlsx
+++ b/outputs/Login-Test-Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R18073f1d7e2f4bf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R00234e24e58f4325"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -551,8 +551,37 @@
         <x:v>artifacts/TC06.png; Allure/TC06</x:v>
       </x:c>
     </x:row>
+    <x:row r="13" ht="66" customHeight="1">
+      <x:c r="A13" s="9" t="str">
+        <x:v>TC07</x:v>
+      </x:c>
+      <x:c r="B13" s="9" t="str">
+        <x:v>Chuyển từ username sang password bằng Tab</x:v>
+      </x:c>
+      <x:c r="C13" s="9" t="str">
+        <x:v>utc_automation_nonexistent_6451071050</x:v>
+      </x:c>
+      <x:c r="D13" s="9" t="str">
+        <x:v>(trống)</x:v>
+      </x:c>
+      <x:c r="E13" s="9" t="str">
+        <x:v>1. Click username. 2. Nhập dữ liệu giả. 3. Nhấn Tab. 4. Kiểm tra focus ở password.</x:v>
+      </x:c>
+      <x:c r="F13" s="9" t="str">
+        <x:v>Tab từ username chuyển focus sang password; username không bị thay đổi.</x:v>
+      </x:c>
+      <x:c r="G13" s="9" t="str">
+        <x:v>BLOCKED</x:v>
+      </x:c>
+      <x:c r="H13" s="9" t="str">
+        <x:v>Không hoàn tất test, exit=2</x:v>
+      </x:c>
+      <x:c r="I13" s="9" t="str">
+        <x:v>artifacts/TC07.png; Allure/TC07</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G7:G12">
+  <x:conditionalFormatting sqref="G7:G13">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="FAIL"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
test(login): TC08 Submit đăng nhập bằng phím Enter (PASS)
</commit_message>
<xml_diff>
--- a/outputs/Login-Test-Cases.xlsx
+++ b/outputs/Login-Test-Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R00234e24e58f4325"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="Rfc98e39f075d47e4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -580,8 +580,37 @@
         <x:v>artifacts/TC07.png; Allure/TC07</x:v>
       </x:c>
     </x:row>
+    <x:row r="14" ht="66" customHeight="1">
+      <x:c r="A14" s="9" t="str">
+        <x:v>TC08</x:v>
+      </x:c>
+      <x:c r="B14" s="9" t="str">
+        <x:v>Submit đăng nhập bằng phím Enter</x:v>
+      </x:c>
+      <x:c r="C14" s="9" t="str">
+        <x:v>utc_automation_nonexistent_6451071050</x:v>
+      </x:c>
+      <x:c r="D14" s="9" t="str">
+        <x:v>Utc_Test_Invalid_2026!</x:v>
+      </x:c>
+      <x:c r="E14" s="9" t="str">
+        <x:v>1. Nhập tài khoản giả. 2. Nhấn Enter trong ô mật khẩu. 3. Kiểm tra response.</x:v>
+      </x:c>
+      <x:c r="F14" s="9" t="str">
+        <x:v>Enter submit form; ở lại Login và báo tài khoản hoặc mật khẩu không đúng.</x:v>
+      </x:c>
+      <x:c r="G14" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H14" s="9" t="str">
+        <x:v>Tài khoản hoặc mật khẩu không đúng.</x:v>
+      </x:c>
+      <x:c r="I14" s="9" t="str">
+        <x:v>artifacts/TC08.png; Allure/TC08</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G7:G13">
+  <x:conditionalFormatting sqref="G7:G14">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="FAIL"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
test(login): TC09 Từ chối dữ liệu chỉ có khoảng trắng (PASS)
</commit_message>
<xml_diff>
--- a/outputs/Login-Test-Cases.xlsx
+++ b/outputs/Login-Test-Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="Rfc98e39f075d47e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R6e2d800e0dfc439a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -609,8 +609,37 @@
         <x:v>artifacts/TC08.png; Allure/TC08</x:v>
       </x:c>
     </x:row>
+    <x:row r="15" ht="66" customHeight="1">
+      <x:c r="A15" s="9" t="str">
+        <x:v>TC09</x:v>
+      </x:c>
+      <x:c r="B15" s="9" t="str">
+        <x:v>Từ chối dữ liệu chỉ có khoảng trắng</x:v>
+      </x:c>
+      <x:c r="C15" s="9" t="str">
+        <x:v>   </x:v>
+      </x:c>
+      <x:c r="D15" s="9" t="str">
+        <x:v>   </x:v>
+      </x:c>
+      <x:c r="E15" s="9" t="str">
+        <x:v>1. Nhập ba dấu cách vào mỗi ô. 2. Nhấn Đăng nhập. 3. Kiểm tra từ chối.</x:v>
+      </x:c>
+      <x:c r="F15" s="9" t="str">
+        <x:v>Không đăng nhập; ở lại Login và có thông báo yêu cầu dữ liệu hoặc thông tin sai.</x:v>
+      </x:c>
+      <x:c r="G15" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H15" s="9" t="str">
+        <x:v>Tài khoản hoặc mật khẩu không đúng.</x:v>
+      </x:c>
+      <x:c r="I15" s="9" t="str">
+        <x:v>artifacts/TC09.png; Allure/TC09</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G7:G14">
+  <x:conditionalFormatting sqref="G7:G15">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="FAIL"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
test(login): TC10 Từ chối username Unicode không tồn tại (BLOCKED)
</commit_message>
<xml_diff>
--- a/outputs/Login-Test-Cases.xlsx
+++ b/outputs/Login-Test-Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R6e2d800e0dfc439a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="Rc3c57f46cb024ad8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -638,8 +638,37 @@
         <x:v>artifacts/TC09.png; Allure/TC09</x:v>
       </x:c>
     </x:row>
+    <x:row r="16" ht="66" customHeight="1">
+      <x:c r="A16" s="9" t="str">
+        <x:v>TC10</x:v>
+      </x:c>
+      <x:c r="B16" s="9" t="str">
+        <x:v>Từ chối username Unicode không tồn tại</x:v>
+      </x:c>
+      <x:c r="C16" s="9" t="str">
+        <x:v>utc_kiểm_thử_không_tồn_tại_6451071050</x:v>
+      </x:c>
+      <x:c r="D16" s="9" t="str">
+        <x:v>Utc_Test_Invalid_2026!</x:v>
+      </x:c>
+      <x:c r="E16" s="9" t="str">
+        <x:v>1. Nhập username giả có dấu tiếng Việt. 2. Nhập password giả. 3. Submit.</x:v>
+      </x:c>
+      <x:c r="F16" s="9" t="str">
+        <x:v>Không đăng nhập; hiển thị thông báo tài khoản hoặc mật khẩu không đúng.</x:v>
+      </x:c>
+      <x:c r="G16" s="9" t="str">
+        <x:v>BLOCKED</x:v>
+      </x:c>
+      <x:c r="H16" s="9" t="str">
+        <x:v>Không hoàn tất test, exit=1</x:v>
+      </x:c>
+      <x:c r="I16" s="9" t="str">
+        <x:v>artifacts/TC10.png; Allure/TC10</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G7:G15">
+  <x:conditionalFormatting sqref="G7:G16">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="FAIL"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
test(login): TC11 Mở trang quên mật khẩu từ login (BLOCKED)
</commit_message>
<xml_diff>
--- a/outputs/Login-Test-Cases.xlsx
+++ b/outputs/Login-Test-Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="Rc3c57f46cb024ad8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R957e37129c624589"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -667,8 +667,37 @@
         <x:v>artifacts/TC10.png; Allure/TC10</x:v>
       </x:c>
     </x:row>
+    <x:row r="17" ht="66" customHeight="1">
+      <x:c r="A17" s="9" t="str">
+        <x:v>TC11</x:v>
+      </x:c>
+      <x:c r="B17" s="9" t="str">
+        <x:v>Mở trang quên mật khẩu từ login</x:v>
+      </x:c>
+      <x:c r="C17" s="9" t="str">
+        <x:v>(trống)</x:v>
+      </x:c>
+      <x:c r="D17" s="9" t="str">
+        <x:v>(trống)</x:v>
+      </x:c>
+      <x:c r="E17" s="9" t="str">
+        <x:v>1. Click link quên mật khẩu. 2. Kiểm tra URL, tiêu đề và ô email/captcha. Không gửi yêu cầu.</x:v>
+      </x:c>
+      <x:c r="F17" s="9" t="str">
+        <x:v>Mở /Login/GetPass, tiêu đề Lấy lại mật khẩu, hiển thị email và captcha.</x:v>
+      </x:c>
+      <x:c r="G17" s="9" t="str">
+        <x:v>BLOCKED</x:v>
+      </x:c>
+      <x:c r="H17" s="9" t="str">
+        <x:v>Không hoàn tất test, exit=1</x:v>
+      </x:c>
+      <x:c r="I17" s="9" t="str">
+        <x:v>artifacts/TC11.png; Allure/TC11</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G7:G16">
+  <x:conditionalFormatting sqref="G7:G17">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="FAIL"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
test(login): TC12 Kiểm tra liên kết đăng nhập e-mail UTC (BLOCKED)
</commit_message>
<xml_diff>
--- a/outputs/Login-Test-Cases.xlsx
+++ b/outputs/Login-Test-Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R957e37129c624589"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R04ea85bf51c5444f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -696,8 +696,37 @@
         <x:v>artifacts/TC11.png; Allure/TC11</x:v>
       </x:c>
     </x:row>
+    <x:row r="18" ht="66" customHeight="1">
+      <x:c r="A18" s="9" t="str">
+        <x:v>TC12</x:v>
+      </x:c>
+      <x:c r="B18" s="9" t="str">
+        <x:v>Kiểm tra liên kết đăng nhập e-mail UTC</x:v>
+      </x:c>
+      <x:c r="C18" s="9" t="str">
+        <x:v>(trống)</x:v>
+      </x:c>
+      <x:c r="D18" s="9" t="str">
+        <x:v>(trống)</x:v>
+      </x:c>
+      <x:c r="E18" s="9" t="str">
+        <x:v>1. Kiểm tra nút đăng nhập e-mail UTC. 2. Đọc URL OAuth và callback. Không mở Google.</x:v>
+      </x:c>
+      <x:c r="F18" s="9" t="str">
+        <x:v>Link hiển thị, trỏ tới HTTPS accounts.google.com, có client_id, response_type=code và callback /Login đúng domain UTC.</x:v>
+      </x:c>
+      <x:c r="G18" s="9" t="str">
+        <x:v>BLOCKED</x:v>
+      </x:c>
+      <x:c r="H18" s="9" t="str">
+        <x:v>Không hoàn tất test, exit=1</x:v>
+      </x:c>
+      <x:c r="I18" s="9" t="str">
+        <x:v>artifacts/TC12.png; Allure/TC12</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G7:G17">
+  <x:conditionalFormatting sqref="G7:G18">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="FAIL"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
test(login): TC13 Quay lại login từ trang quên mật khẩu (PASS)
</commit_message>
<xml_diff>
--- a/outputs/Login-Test-Cases.xlsx
+++ b/outputs/Login-Test-Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R04ea85bf51c5444f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="Radba91058bab4814"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -725,8 +725,37 @@
         <x:v>artifacts/TC12.png; Allure/TC12</x:v>
       </x:c>
     </x:row>
+    <x:row r="19" ht="66" customHeight="1">
+      <x:c r="A19" s="9" t="str">
+        <x:v>TC13</x:v>
+      </x:c>
+      <x:c r="B19" s="9" t="str">
+        <x:v>Quay lại login từ trang quên mật khẩu</x:v>
+      </x:c>
+      <x:c r="C19" s="9" t="str">
+        <x:v>(trống)</x:v>
+      </x:c>
+      <x:c r="D19" s="9" t="str">
+        <x:v>(trống)</x:v>
+      </x:c>
+      <x:c r="E19" s="9" t="str">
+        <x:v>1. Mở quên mật khẩu. 2. Click Trở lại đăng nhập. 3. Kiểm tra form login.</x:v>
+      </x:c>
+      <x:c r="F19" s="9" t="str">
+        <x:v>Quay về /Login, ô username và password cùng nút đăng nhập hiển thị.</x:v>
+      </x:c>
+      <x:c r="G19" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H19" s="9" t="str">
+        <x:v>Đã chạy trên Chrome hiển thị; các assertion đạt.</x:v>
+      </x:c>
+      <x:c r="I19" s="9" t="str">
+        <x:v>artifacts/TC13.png; Allure/TC13</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G7:G18">
+  <x:conditionalFormatting sqref="G7:G19">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="FAIL"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
test(login): TC14 Thử lại sau lỗi thiếu mật khẩu (PASS)
</commit_message>
<xml_diff>
--- a/outputs/Login-Test-Cases.xlsx
+++ b/outputs/Login-Test-Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="Radba91058bab4814"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R9eaaa45f189744e9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -754,8 +754,37 @@
         <x:v>artifacts/TC13.png; Allure/TC13</x:v>
       </x:c>
     </x:row>
+    <x:row r="20" ht="66" customHeight="1">
+      <x:c r="A20" s="9" t="str">
+        <x:v>TC14</x:v>
+      </x:c>
+      <x:c r="B20" s="9" t="str">
+        <x:v>Thử lại sau lỗi thiếu mật khẩu</x:v>
+      </x:c>
+      <x:c r="C20" s="9" t="str">
+        <x:v>utc_automation_nonexistent_6451071050</x:v>
+      </x:c>
+      <x:c r="D20" s="9" t="str">
+        <x:v>Utc_Test_Invalid_2026!</x:v>
+      </x:c>
+      <x:c r="E20" s="9" t="str">
+        <x:v>1. Submit chỉ có username giả. 2. Kiểm tra lỗi thiếu mật khẩu. 3. Nhập đủ dữ liệu giả và submit lại. 4. Kiểm tra thông báo mới.</x:v>
+      </x:c>
+      <x:c r="F20" s="9" t="str">
+        <x:v>Lượt đầu báo chưa nhập mật khẩu; lượt sau báo tài khoản hoặc mật khẩu không đúng và không còn lỗi thiếu mật khẩu.</x:v>
+      </x:c>
+      <x:c r="G20" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H20" s="9" t="str">
+        <x:v>Tài khoản hoặc mật khẩu không đúng.</x:v>
+      </x:c>
+      <x:c r="I20" s="9" t="str">
+        <x:v>artifacts/TC14.png; Allure/TC14</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G7:G19">
+  <x:conditionalFormatting sqref="G7:G20">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="FAIL"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
docs: record 14-case coverage and final passing regression results
</commit_message>
<xml_diff>
--- a/outputs/Login-Test-Cases.xlsx
+++ b/outputs/Login-Test-Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R9eaaa45f189744e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Test Cases" sheetId="1" r:id="R5482e83e9b2940d5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -571,10 +571,10 @@
         <x:v>Tab từ username chuyển focus sang password; username không bị thay đổi.</x:v>
       </x:c>
       <x:c r="G13" s="9" t="str">
-        <x:v>BLOCKED</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="H13" s="9" t="str">
-        <x:v>Không hoàn tất test, exit=2</x:v>
+        <x:v>Đã chạy trên Chrome hiển thị; các assertion đạt.</x:v>
       </x:c>
       <x:c r="I13" s="9" t="str">
         <x:v>artifacts/TC07.png; Allure/TC07</x:v>
@@ -617,10 +617,10 @@
         <x:v>Từ chối dữ liệu chỉ có khoảng trắng</x:v>
       </x:c>
       <x:c r="C15" s="9" t="str">
-        <x:v>   </x:v>
+        <x:v>(3 dấu cách)</x:v>
       </x:c>
       <x:c r="D15" s="9" t="str">
-        <x:v>   </x:v>
+        <x:v>(3 dấu cách)</x:v>
       </x:c>
       <x:c r="E15" s="9" t="str">
         <x:v>1. Nhập ba dấu cách vào mỗi ô. 2. Nhấn Đăng nhập. 3. Kiểm tra từ chối.</x:v>
@@ -658,10 +658,10 @@
         <x:v>Không đăng nhập; hiển thị thông báo tài khoản hoặc mật khẩu không đúng.</x:v>
       </x:c>
       <x:c r="G16" s="9" t="str">
-        <x:v>BLOCKED</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="H16" s="9" t="str">
-        <x:v>Không hoàn tất test, exit=1</x:v>
+        <x:v>Tài khoản hoặc mật khẩu không đúng.</x:v>
       </x:c>
       <x:c r="I16" s="9" t="str">
         <x:v>artifacts/TC10.png; Allure/TC10</x:v>
@@ -687,10 +687,10 @@
         <x:v>Mở /Login/GetPass, tiêu đề Lấy lại mật khẩu, hiển thị email và captcha.</x:v>
       </x:c>
       <x:c r="G17" s="9" t="str">
-        <x:v>BLOCKED</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="H17" s="9" t="str">
-        <x:v>Không hoàn tất test, exit=1</x:v>
+        <x:v>Đã chạy trên Chrome hiển thị; các assertion đạt.</x:v>
       </x:c>
       <x:c r="I17" s="9" t="str">
         <x:v>artifacts/TC11.png; Allure/TC11</x:v>
@@ -716,10 +716,10 @@
         <x:v>Link hiển thị, trỏ tới HTTPS accounts.google.com, có client_id, response_type=code và callback /Login đúng domain UTC.</x:v>
       </x:c>
       <x:c r="G18" s="9" t="str">
-        <x:v>BLOCKED</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="H18" s="9" t="str">
-        <x:v>Không hoàn tất test, exit=1</x:v>
+        <x:v>Đã chạy trên Chrome hiển thị; các assertion đạt.</x:v>
       </x:c>
       <x:c r="I18" s="9" t="str">
         <x:v>artifacts/TC12.png; Allure/TC12</x:v>

</xml_diff>